<commit_message>
projet amélioré pour la recherche par dates, d'autres améliorations à rajouter pour un fonctionnement optimal
</commit_message>
<xml_diff>
--- a/data/04_testVectorisation/QuestionTest.xlsx
+++ b/data/04_testVectorisation/QuestionTest.xlsx
@@ -468,7 +468,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>quel évènement se sont produit le 25 août 2025 à Nice ?</t>
+          <t>quels évènements se sont produit le 25 août 2025 à Nice ?</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -483,12 +483,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>94917451-6 : none - 78337946 : none</t>
+          <t>94917451-6 : none - 78337946 : 28</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>94917451-6 : none - 78337946 : none</t>
+          <t>94917451-6 : none - 78337946 : 83.37268233299255</t>
         </is>
       </c>
     </row>
@@ -515,12 +515,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>76804754 : 1 - 6940499 : 2</t>
+          <t>76804754 : 2 - 6940499 : 1</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>76804754 : 84.77242588996887 - 6940499 : 84.77242588996887</t>
+          <t>76804754 : 84.89689826965332 - 6940499 : 84.89689826965332</t>
         </is>
       </c>
     </row>
@@ -547,12 +547,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>76804754 : 1 - 6940499 : 2</t>
+          <t>76804754 : 2 - 6940499 : 1</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>76804754 : 86.70159578323364 - 6940499 : 86.70159578323364</t>
+          <t>76804754 : 87.29822635650635 - 6940499 : 87.29822635650635</t>
         </is>
       </c>
     </row>
@@ -579,12 +579,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>21312701 : 147</t>
+          <t>21312701 : 95</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>21312701 : 81.92882537841797</t>
+          <t>21312701 : 83.05857181549072</t>
         </is>
       </c>
     </row>

</xml_diff>